<commit_message>
Update parts list and remove old one
</commit_message>
<xml_diff>
--- a/hardware/parts_list.xlsx
+++ b/hardware/parts_list.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hrobi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hrobi\Desktop\Esp32 PingBox\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{078463E1-1758-425A-BD0F-030593D31BD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB242366-605F-44C5-B7A3-288E267595F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="3810" windowWidth="28800" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts List" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t>Parts List</t>
   </si>
@@ -90,6 +90,61 @@
   </si>
   <si>
     <t>Led button</t>
+  </si>
+  <si>
+    <t>⚠️ Late-Addition Components</t>
+  </si>
+  <si>
+    <t>Why it was added</t>
+  </si>
+  <si>
+    <t>Buck Converter LM2596</t>
+  </si>
+  <si>
+    <t>USB C Male Pigtail Cable</t>
+  </si>
+  <si>
+    <t>⚠️ Added after expansion board failure - see README</t>
+  </si>
+  <si>
+    <t>These parts were added mid-project. Full context in README.md</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">--&gt; Use </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>9V</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> !    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Or else --&gt;</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -99,7 +154,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -147,8 +202,60 @@
       <color rgb="FF2E75B6"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FF7F6000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF7F6000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -175,8 +282,29 @@
         <fgColor rgb="FFD6E4F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7F6000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFDE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFDE7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -214,11 +342,68 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFBF8F00"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFBF8F00"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFBF8F00"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBF8F00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBF8F00"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBF8F00"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBF8F00"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBF8F00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBF8F00"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBF8F00"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBF8F00"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBF8F00"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBF8F00"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBF8F00"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -264,12 +449,38 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFF2CC"/>
+      <color rgb="FFFFFDE7"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -566,23 +777,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:E16"/>
+  <dimension ref="B1:I16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
     <col min="4" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="22.85546875" customWidth="1"/>
+    <col min="7" max="7" width="29.85546875" customWidth="1"/>
+    <col min="8" max="8" width="31.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:9" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" s="15" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="16"/>
       <c r="D1" s="16"/>
       <c r="E1" s="16"/>
-    </row>
-    <row r="2" spans="2:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G1" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="H1" s="16"/>
+    </row>
+    <row r="2" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
@@ -595,8 +813,12 @@
       <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G2" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" s="16"/>
+    </row>
+    <row r="3" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -609,8 +831,17 @@
       <c r="E3" s="4">
         <v>6.3</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G3" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
         <v>5</v>
       </c>
@@ -623,8 +854,17 @@
       <c r="E4" s="7">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G4" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="4">
+        <v>1.71</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>6</v>
       </c>
@@ -637,8 +877,18 @@
       <c r="E5" s="4">
         <v>2.5</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F5" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="22"/>
+      <c r="I5" s="4">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>18</v>
       </c>
@@ -652,7 +902,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="7" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
@@ -666,7 +916,7 @@
         <v>1.55</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>8</v>
       </c>
@@ -680,7 +930,7 @@
         <v>2.81</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>9</v>
       </c>
@@ -694,7 +944,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="5" t="s">
         <v>10</v>
       </c>
@@ -708,7 +958,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="11" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
         <v>11</v>
       </c>
@@ -722,7 +972,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="12" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="5" t="s">
         <v>12</v>
       </c>
@@ -736,7 +986,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="13" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
         <v>13</v>
       </c>
@@ -744,7 +994,7 @@
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
     </row>
-    <row r="14" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
         <v>14</v>
       </c>
@@ -752,7 +1002,7 @@
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
     </row>
-    <row r="15" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
         <v>15</v>
       </c>
@@ -764,7 +1014,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="12" t="s">
         <v>16</v>
       </c>
@@ -779,8 +1029,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="4">
     <mergeCell ref="B1:E1"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="H4:H5"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -793,6 +1046,8 @@
     <hyperlink ref="B10" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
     <hyperlink ref="B11" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="B12" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="G5" r:id="rId11" xr:uid="{D44F927E-5286-4D4B-80A5-3F02AC68C21F}"/>
+    <hyperlink ref="G4" r:id="rId12" xr:uid="{58263611-9F58-449D-8E31-6BBA51F21DCB}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>